<commit_message>
rigor: add real weather and sensitivity analysis
</commit_message>
<xml_diff>
--- a/outputs/submission/q3_vehicle_allocation.xlsx
+++ b/outputs/submission/q3_vehicle_allocation.xlsx
@@ -615,10 +615,10 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>0.7861391375372468</v>
+        <v>0.745565033370428</v>
       </c>
       <c r="D2">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E2">
         <v>17.80434782608696</v>
@@ -630,7 +630,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -641,10 +641,10 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>7.322297995673891</v>
+        <v>7.341706281548541</v>
       </c>
       <c r="D3">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E3">
         <v>17.80434782608696</v>
@@ -667,10 +667,10 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>11.62018561329523</v>
+        <v>12.20216708574654</v>
       </c>
       <c r="D4">
-        <v>5.754416666666667</v>
+        <v>5.601083333333334</v>
       </c>
       <c r="E4">
         <v>17.96111111111111</v>
@@ -693,10 +693,10 @@
         <v>11</v>
       </c>
       <c r="C5">
-        <v>2.799648386947021</v>
+        <v>2.822701005736524</v>
       </c>
       <c r="D5">
-        <v>2.983000000000001</v>
+        <v>2.993000000000001</v>
       </c>
       <c r="E5">
         <v>8.933333333333334</v>
@@ -719,10 +719,10 @@
         <v>12</v>
       </c>
       <c r="C6">
-        <v>6.111878476579959</v>
+        <v>6.465768028453207</v>
       </c>
       <c r="D6">
-        <v>3.469250000000001</v>
+        <v>3.47925</v>
       </c>
       <c r="E6">
         <v>23.23333333333333</v>
@@ -745,10 +745,10 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>24.88262106655043</v>
+        <v>25.9600841186291</v>
       </c>
       <c r="D7">
-        <v>5.055333333333334</v>
+        <v>5.002000000000001</v>
       </c>
       <c r="E7">
         <v>15.38333333333333</v>
@@ -771,10 +771,10 @@
         <v>14</v>
       </c>
       <c r="C8">
-        <v>6.03180130520032</v>
+        <v>6.098383669369557</v>
       </c>
       <c r="D8">
-        <v>4.59975</v>
+        <v>4.639750000000001</v>
       </c>
       <c r="E8">
         <v>9.733333333333333</v>
@@ -797,10 +797,10 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>4.464689909067117</v>
+        <v>4.618268197974807</v>
       </c>
       <c r="D9">
-        <v>2.163</v>
+        <v>2.213</v>
       </c>
       <c r="E9">
         <v>7.55</v>
@@ -823,10 +823,10 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>37.44260923368128</v>
+        <v>38.50316475293453</v>
       </c>
       <c r="D10">
-        <v>14.96212500000001</v>
+        <v>15.32712500000001</v>
       </c>
       <c r="E10">
         <v>50.09166666666666</v>
@@ -835,10 +835,10 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H10">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -849,10 +849,10 @@
         <v>17</v>
       </c>
       <c r="C11">
-        <v>0.2537254417051208</v>
+        <v>0.240586001509577</v>
       </c>
       <c r="D11">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E11">
         <v>17.80434782608696</v>
@@ -875,10 +875,10 @@
         <v>18</v>
       </c>
       <c r="C12">
-        <v>5.739968902964273</v>
+        <v>5.792965279038185</v>
       </c>
       <c r="D12">
-        <v>2.571333333333334</v>
+        <v>2.404666666666667</v>
       </c>
       <c r="E12">
         <v>6.566666666666666</v>
@@ -901,10 +901,10 @@
         <v>19</v>
       </c>
       <c r="C13">
-        <v>2.73577192652567</v>
+        <v>2.557964414033694</v>
       </c>
       <c r="D13">
-        <v>4.054666666666667</v>
+        <v>4.128</v>
       </c>
       <c r="E13">
         <v>12.04444444444444</v>
@@ -927,10 +927,10 @@
         <v>20</v>
       </c>
       <c r="C14">
-        <v>4.521404831642053</v>
+        <v>4.539136458158642</v>
       </c>
       <c r="D14">
-        <v>6.142308899592942</v>
+        <v>6.206058899592942</v>
       </c>
       <c r="E14">
         <v>23.7875</v>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
         <v>2</v>
@@ -953,10 +953,10 @@
         <v>21</v>
       </c>
       <c r="C15">
-        <v>7.009948831877653</v>
+        <v>7.028618253948109</v>
       </c>
       <c r="D15">
-        <v>3.94175</v>
+        <v>3.849250000000001</v>
       </c>
       <c r="E15">
         <v>11.8375</v>
@@ -979,10 +979,10 @@
         <v>22</v>
       </c>
       <c r="C16">
-        <v>8.645191346491213</v>
+        <v>9.149581663248799</v>
       </c>
       <c r="D16">
-        <v>7.484125</v>
+        <v>7.459125000000001</v>
       </c>
       <c r="E16">
         <v>24.88333333333333</v>
@@ -1005,10 +1005,10 @@
         <v>23</v>
       </c>
       <c r="C17">
-        <v>7.954193931385616</v>
+        <v>7.975525574990453</v>
       </c>
       <c r="D17">
-        <v>7.030000000000001</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="E17">
         <v>30.38333333333333</v>
@@ -1031,10 +1031,10 @@
         <v>24</v>
       </c>
       <c r="C18">
-        <v>13.94925417228803</v>
+        <v>14.45065491706647</v>
       </c>
       <c r="D18">
-        <v>3.294</v>
+        <v>3.274000000000001</v>
       </c>
       <c r="E18">
         <v>11.7</v>
@@ -1057,10 +1057,10 @@
         <v>25</v>
       </c>
       <c r="C19">
-        <v>0.8685782852997461</v>
+        <v>0.8373578803924049</v>
       </c>
       <c r="D19">
-        <v>3.487710440003781</v>
+        <v>3.567710440003781</v>
       </c>
       <c r="E19">
         <v>7.316666666666666</v>
@@ -1083,10 +1083,10 @@
         <v>26</v>
       </c>
       <c r="C20">
-        <v>4.288708031910989</v>
+        <v>4.173798336670656</v>
       </c>
       <c r="D20">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E20">
         <v>17.80434782608696</v>
@@ -1109,10 +1109,10 @@
         <v>27</v>
       </c>
       <c r="C21">
-        <v>15.45759622151422</v>
+        <v>15.93391957515696</v>
       </c>
       <c r="D21">
-        <v>4.196464285714286</v>
+        <v>4.232178571428571</v>
       </c>
       <c r="E21">
         <v>15.15714285714286</v>
@@ -1121,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H21">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1135,10 +1135,10 @@
         <v>28</v>
       </c>
       <c r="C22">
-        <v>3.97514743887</v>
+        <v>3.897183612393216</v>
       </c>
       <c r="D22">
-        <v>4.961000000000002</v>
+        <v>4.891000000000002</v>
       </c>
       <c r="E22">
         <v>22.81666666666666</v>
@@ -1161,10 +1161,10 @@
         <v>29</v>
       </c>
       <c r="C23">
-        <v>1.994669731576661</v>
+        <v>1.983265885217715</v>
       </c>
       <c r="D23">
-        <v>6.708374999999999</v>
+        <v>6.973375</v>
       </c>
       <c r="E23">
         <v>18.74166666666666</v>
@@ -1187,10 +1187,10 @@
         <v>30</v>
       </c>
       <c r="C24">
-        <v>32.76761727819967</v>
+        <v>33.66430664474652</v>
       </c>
       <c r="D24">
-        <v>13.04822738512074</v>
+        <v>13.66222738512074</v>
       </c>
       <c r="E24">
         <v>19.79</v>
@@ -1202,7 +1202,7 @@
         <v>11</v>
       </c>
       <c r="H24">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1213,10 +1213,10 @@
         <v>31</v>
       </c>
       <c r="C25">
-        <v>11.82052560370878</v>
+        <v>12.52841222415983</v>
       </c>
       <c r="D25">
-        <v>3.2775</v>
+        <v>3.2675</v>
       </c>
       <c r="E25">
         <v>10.93333333333333</v>
@@ -1239,10 +1239,10 @@
         <v>32</v>
       </c>
       <c r="C26">
-        <v>1.478455497664508</v>
+        <v>1.468197958233695</v>
       </c>
       <c r="D26">
-        <v>2.661500000000001</v>
+        <v>2.731500000000001</v>
       </c>
       <c r="E26">
         <v>8.966666666666667</v>
@@ -1265,10 +1265,10 @@
         <v>33</v>
       </c>
       <c r="C27">
-        <v>5.353767491539864</v>
+        <v>5.363602807817085</v>
       </c>
       <c r="D27">
-        <v>6.577000000000005</v>
+        <v>6.527000000000005</v>
       </c>
       <c r="E27">
         <v>46.66666666666666</v>
@@ -1291,10 +1291,10 @@
         <v>34</v>
       </c>
       <c r="C28">
-        <v>5.375049907722471</v>
+        <v>5.711714589658509</v>
       </c>
       <c r="D28">
-        <v>2.6385</v>
+        <v>2.7185</v>
       </c>
       <c r="E28">
         <v>6.616666666666666</v>
@@ -1317,10 +1317,10 @@
         <v>35</v>
       </c>
       <c r="C29">
-        <v>12.91545612174226</v>
+        <v>13.47745784217993</v>
       </c>
       <c r="D29">
-        <v>7.1330625</v>
+        <v>7.3655625</v>
       </c>
       <c r="E29">
         <v>18.9375</v>
@@ -1343,10 +1343,10 @@
         <v>36</v>
       </c>
       <c r="C30">
-        <v>2.615911845230452</v>
+        <v>2.59776127746782</v>
       </c>
       <c r="D30">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E30">
         <v>17.80434782608696</v>
@@ -1369,10 +1369,10 @@
         <v>37</v>
       </c>
       <c r="C31">
-        <v>3.079408534455307</v>
+        <v>3.008073829269156</v>
       </c>
       <c r="D31">
-        <v>5.132375000000001</v>
+        <v>5.095708333333334</v>
       </c>
       <c r="E31">
         <v>16.21388888888889</v>
@@ -1381,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -1395,10 +1395,10 @@
         <v>38</v>
       </c>
       <c r="C32">
-        <v>5.810112964203543</v>
+        <v>6.042475914545943</v>
       </c>
       <c r="D32">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E32">
         <v>17.80434782608696</v>
@@ -1421,10 +1421,10 @@
         <v>39</v>
       </c>
       <c r="C33">
-        <v>8.205891985075061</v>
+        <v>8.273337985917321</v>
       </c>
       <c r="D33">
-        <v>3.788666666666667</v>
+        <v>3.748666666666667</v>
       </c>
       <c r="E33">
         <v>10.98333333333333</v>
@@ -1447,10 +1447,10 @@
         <v>40</v>
       </c>
       <c r="C34">
-        <v>6.169885853583731</v>
+        <v>6.206073151157904</v>
       </c>
       <c r="D34">
-        <v>5.3245</v>
+        <v>5.3995</v>
       </c>
       <c r="E34">
         <v>17.625</v>
@@ -1473,10 +1473,10 @@
         <v>41</v>
       </c>
       <c r="C35">
-        <v>28.49746097978402</v>
+        <v>29.83121606480299</v>
       </c>
       <c r="D35">
-        <v>4.272000000000001</v>
+        <v>4.262</v>
       </c>
       <c r="E35">
         <v>13.15833333333333</v>
@@ -1499,10 +1499,10 @@
         <v>42</v>
       </c>
       <c r="C36">
-        <v>2.681151403454418</v>
+        <v>2.622867715503946</v>
       </c>
       <c r="D36">
-        <v>4.113999999999999</v>
+        <v>4.154</v>
       </c>
       <c r="E36">
         <v>13.28333333333333</v>
@@ -1525,10 +1525,10 @@
         <v>43</v>
       </c>
       <c r="C37">
-        <v>3.379638607354134</v>
+        <v>3.441056130829438</v>
       </c>
       <c r="D37">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E37">
         <v>17.80434782608696</v>
@@ -1551,10 +1551,10 @@
         <v>44</v>
       </c>
       <c r="C38">
-        <v>0.0282952973987074</v>
+        <v>0.0274674365258816</v>
       </c>
       <c r="D38">
-        <v>2.956499999999999</v>
+        <v>2.886499999999999</v>
       </c>
       <c r="E38">
         <v>5.383333333333334</v>
@@ -1577,10 +1577,10 @@
         <v>45</v>
       </c>
       <c r="C39">
-        <v>3.786251342058054</v>
+        <v>3.825339677968438</v>
       </c>
       <c r="D39">
-        <v>6.436496553227734</v>
+        <v>6.376496553227734</v>
       </c>
       <c r="E39">
         <v>28.1</v>
@@ -1603,10 +1603,10 @@
         <v>46</v>
       </c>
       <c r="C40">
-        <v>3.582216156420516</v>
+        <v>3.572505789499097</v>
       </c>
       <c r="D40">
-        <v>4.6645</v>
+        <v>4.5845</v>
       </c>
       <c r="E40">
         <v>9.816666666666666</v>
@@ -1629,10 +1629,10 @@
         <v>47</v>
       </c>
       <c r="C41">
-        <v>2.750618823692184</v>
+        <v>2.767953938427828</v>
       </c>
       <c r="D41">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E41">
         <v>17.80434782608696</v>
@@ -1655,10 +1655,10 @@
         <v>48</v>
       </c>
       <c r="C42">
-        <v>3.296808397313321</v>
+        <v>3.368600458684325</v>
       </c>
       <c r="D42">
-        <v>12.09005834215038</v>
+        <v>11.91672500881705</v>
       </c>
       <c r="E42">
         <v>24.33333333333333</v>
@@ -1681,10 +1681,10 @@
         <v>49</v>
       </c>
       <c r="C43">
-        <v>1.516688636481844</v>
+        <v>1.417548789534279</v>
       </c>
       <c r="D43">
-        <v>3.294000000000001</v>
+        <v>3.544000000000001</v>
       </c>
       <c r="E43">
         <v>9.5</v>
@@ -1707,10 +1707,10 @@
         <v>50</v>
       </c>
       <c r="C44">
-        <v>0.1954610306881022</v>
+        <v>0.197328374047944</v>
       </c>
       <c r="D44">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E44">
         <v>17.80434782608696</v>
@@ -1733,10 +1733,10 @@
         <v>51</v>
       </c>
       <c r="C45">
-        <v>3.313539259191428</v>
+        <v>3.154745087805411</v>
       </c>
       <c r="D45">
-        <v>3.723500000000002</v>
+        <v>3.693500000000002</v>
       </c>
       <c r="E45">
         <v>7.466666666666667</v>
@@ -1759,10 +1759,10 @@
         <v>52</v>
       </c>
       <c r="C46">
-        <v>6.700600198584287</v>
+        <v>6.752419312739973</v>
       </c>
       <c r="D46">
-        <v>5.2845</v>
+        <v>5.3345</v>
       </c>
       <c r="E46">
         <v>13.11666666666667</v>
@@ -1785,10 +1785,10 @@
         <v>53</v>
       </c>
       <c r="C47">
-        <v>3.61777963433221</v>
+        <v>3.594886018975857</v>
       </c>
       <c r="D47">
-        <v>7.228875</v>
+        <v>7.288875000000001</v>
       </c>
       <c r="E47">
         <v>29.49166666666667</v>
@@ -1811,10 +1811,10 @@
         <v>54</v>
       </c>
       <c r="C48">
-        <v>2.120760123483058</v>
+        <v>2.12592852023809</v>
       </c>
       <c r="D48">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E48">
         <v>17.80434782608696</v>
@@ -1837,10 +1837,10 @@
         <v>55</v>
       </c>
       <c r="C49">
-        <v>23.40172630842621</v>
+        <v>25.66391557713383</v>
       </c>
       <c r="D49">
-        <v>3.898277777777778</v>
+        <v>3.879388888888889</v>
       </c>
       <c r="E49">
         <v>9.633333333333333</v>
@@ -1852,7 +1852,7 @@
         <v>4</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -1863,10 +1863,10 @@
         <v>56</v>
       </c>
       <c r="C50">
-        <v>9.526158228192203</v>
+        <v>10.06765522243298</v>
       </c>
       <c r="D50">
-        <v>5.601083333333334</v>
+        <v>5.607749999999999</v>
       </c>
       <c r="E50">
         <v>18.71111111111111</v>
@@ -1878,7 +1878,7 @@
         <v>3</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -1889,10 +1889,10 @@
         <v>57</v>
       </c>
       <c r="C51">
-        <v>5.616671685113239</v>
+        <v>6.092554171704538</v>
       </c>
       <c r="D51">
-        <v>3.640000000000001</v>
+        <v>3.65</v>
       </c>
       <c r="E51">
         <v>11.3</v>
@@ -1915,10 +1915,10 @@
         <v>58</v>
       </c>
       <c r="C52">
-        <v>0.2567070836394975</v>
+        <v>0.2465956337974</v>
       </c>
       <c r="D52">
-        <v>5.80866537068958</v>
+        <v>5.849361022863494</v>
       </c>
       <c r="E52">
         <v>17.80434782608696</v>
@@ -1941,10 +1941,10 @@
         <v>59</v>
       </c>
       <c r="C53">
-        <v>2.372851367464393</v>
+        <v>2.4260424794793</v>
       </c>
       <c r="D53">
-        <v>3.5815</v>
+        <v>3.701500000000001</v>
       </c>
       <c r="E53">
         <v>7.633333333333334</v>
@@ -1967,10 +1967,10 @@
         <v>60</v>
       </c>
       <c r="C54">
-        <v>5.479686822169914</v>
+        <v>5.58336643499782</v>
       </c>
       <c r="D54">
-        <v>2.787</v>
+        <v>2.736999999999999</v>
       </c>
       <c r="E54">
         <v>10.01666666666667</v>
@@ -1993,10 +1993,10 @@
         <v>61</v>
       </c>
       <c r="C55">
-        <v>2.709147007317714</v>
+        <v>2.751724916137945</v>
       </c>
       <c r="D55">
-        <v>8.214499999999997</v>
+        <v>8.204499999999999</v>
       </c>
       <c r="E55">
         <v>28.05</v>
@@ -2019,10 +2019,10 @@
         <v>62</v>
       </c>
       <c r="C56">
-        <v>3.313518313947521</v>
+        <v>3.293675352324498</v>
       </c>
       <c r="D56">
-        <v>15.84678438081632</v>
+        <v>16.93678438081632</v>
       </c>
       <c r="E56">
         <v>83.38333333333334</v>
@@ -2045,10 +2045,10 @@
         <v>63</v>
       </c>
       <c r="C57">
-        <v>7.357317181874623</v>
+        <v>7.65442465999378</v>
       </c>
       <c r="D57">
-        <v>9.132999999999999</v>
+        <v>9.283000000000005</v>
       </c>
       <c r="E57">
         <v>24.81666666666666</v>
@@ -2071,10 +2071,10 @@
         <v>64</v>
       </c>
       <c r="C58">
-        <v>2.699824615211464</v>
+        <v>2.761465361488717</v>
       </c>
       <c r="D58">
-        <v>6.151624999999999</v>
+        <v>6.216625000000001</v>
       </c>
       <c r="E58">
         <v>27.48333333333333</v>
@@ -2097,10 +2097,10 @@
         <v>65</v>
       </c>
       <c r="C59">
-        <v>3.538973155073464</v>
+        <v>3.497788745797252</v>
       </c>
       <c r="D59">
-        <v>6.387499999999999</v>
+        <v>5.7875</v>
       </c>
       <c r="E59">
         <v>16.48333333333333</v>
@@ -2123,10 +2123,10 @@
         <v>66</v>
       </c>
       <c r="C60">
-        <v>3.779102849767777</v>
+        <v>3.744159174953809</v>
       </c>
       <c r="D60">
-        <v>8.342750000000001</v>
+        <v>8.229416666666669</v>
       </c>
       <c r="E60">
         <v>24.08888888888889</v>
@@ -2149,10 +2149,10 @@
         <v>67</v>
       </c>
       <c r="C61">
-        <v>2.389828628283801</v>
+        <v>2.402019694541912</v>
       </c>
       <c r="D61">
-        <v>4.608900000000001</v>
+        <v>4.5869</v>
       </c>
       <c r="E61">
         <v>12.31333333333333</v>
@@ -2175,10 +2175,10 @@
         <v>68</v>
       </c>
       <c r="C62">
-        <v>3.052716971060664</v>
+        <v>3.148642850221658</v>
       </c>
       <c r="D62">
-        <v>4.902</v>
+        <v>4.912</v>
       </c>
       <c r="E62">
         <v>10.93333333333333</v>

</xml_diff>